<commit_message>
Add round 2 to israelis-50-plus-database (5 more verified sports entries, 13 total)
</commit_message>
<xml_diff>
--- a/.claude/skills/israelis-50-plus-database/database.xlsx
+++ b/.claude/skills/israelis-50-plus-database/database.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="81">
   <si>
     <t>שם</t>
   </si>
@@ -164,6 +164,96 @@
   </si>
   <si>
     <t>https://www.ynet.co.il/sport/tokyoparalympics2020/article/bk3tjgowy</t>
+  </si>
+  <si>
+    <t>שמעון סימקין</t>
+  </si>
+  <si>
+    <t>כ-73 (זכה באליפות עולם בגיל 89)</t>
+  </si>
+  <si>
+    <t>שירת כשליח בצבא האדום במלחמת העולם השנייה ולמד לרוץ בשדה הקרב, אך לא התאמן ברצינות שנים רבות</t>
+  </si>
+  <si>
+    <t>התחיל להתאמן ולהתחרות ברצינות בגיל מבוגר, וזכה באליפות העולם לוותיקים בריצת 10 ק"מ (קטגוריית 85+)</t>
+  </si>
+  <si>
+    <t>ריצה (אתלטיקה, ותיקים)</t>
+  </si>
+  <si>
+    <t>https://www.ynet.co.il/articles/0,7340,L-4385741,00.html</t>
+  </si>
+  <si>
+    <t>טטיאנה אברמסון</t>
+  </si>
+  <si>
+    <t>50 (טיפוס ראשון), 55 (הישג השיא)</t>
+  </si>
+  <si>
+    <t>מאמנת התעמלות אמנותית מבאר שבע, גידלה משפחה ולימדה התעמלות, לא טיפסה הרים</t>
+  </si>
+  <si>
+    <t>התחילה בטיפוס קיר בגיל 50, טיפסה את הר מרמולדה, ובגיל 55 הפכה לישראלית הראשונה שטיפסה על הר מאנסלו בהימלאיה (8,163 מ')</t>
+  </si>
+  <si>
+    <t>טיפוס הרים</t>
+  </si>
+  <si>
+    <t>https://www.ynet.co.il/laisha/article/HkpzvrrDO</t>
+  </si>
+  <si>
+    <t>דן הרטנו</t>
+  </si>
+  <si>
+    <t>66 (התחלה), 72 (חגורה שחורה)</t>
+  </si>
+  <si>
+    <t>פיזיותרפיסט מרעננה, ללא רקע באומנויות לחימה</t>
+  </si>
+  <si>
+    <t>התחיל להתאמן קראטה בגיל 66, ובגיל 72 - עם קוצב לב שהושתל שלוש שנים קודם לכן - קיבל חגורה שחורה</t>
+  </si>
+  <si>
+    <t>קראטה</t>
+  </si>
+  <si>
+    <t>https://xnet.ynet.co.il/articles/0,7340,L-5527147,00.html</t>
+  </si>
+  <si>
+    <t>פסקל ברקוביץ</t>
+  </si>
+  <si>
+    <t>55</t>
+  </si>
+  <si>
+    <t>ספורטאית פראלימפית מנוסה (שחייה מגיל 20, חתירה מגיל 40) שאיבדה את רגליה בתאונה בפריז כשהייתה צעירה</t>
+  </si>
+  <si>
+    <t>בגיל 55 עברה לענף הקיאקים (paracanoe) כדי להתחרות במשחקים הפראלימפיים בפריז 2024 - "סגירת מעגל" במקום בו איבדה את רגליה</t>
+  </si>
+  <si>
+    <t>קיאקים פראלימפי (paracanoe)</t>
+  </si>
+  <si>
+    <t>https://www.calcalist.co.il/style/article/b1tj7hswi</t>
+  </si>
+  <si>
+    <t>נעמי רונן</t>
+  </si>
+  <si>
+    <t>לא מאומת במקור - ההישג תועד בגיל 91-92, לא עסקה בספורט קודם לכן</t>
+  </si>
+  <si>
+    <t>"לא עסקה בספורט במשך רוב חייה", לפי הכתבה</t>
+  </si>
+  <si>
+    <t>הוכרה על ידי ספר השיאים של גינס כאישה המבוגרת בעולם שעומדת על הראש; מבצעת גם שכיבות סמיכה ותרגילי כוח</t>
+  </si>
+  <si>
+    <t>התעמלות/כושר גופני</t>
+  </si>
+  <si>
+    <t>https://www.haaretz.co.il/news/local/2025-02-14/ty-article/.premium/00000195-00ec-d1d7-a9d5-f8edb3990000</t>
   </si>
 </sst>
 </file>
@@ -577,7 +667,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -768,6 +858,106 @@
         <v>50</v>
       </c>
     </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>80</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="F2" r:id="rId1"/>
@@ -778,6 +968,11 @@
     <hyperlink ref="F7" r:id="rId6"/>
     <hyperlink ref="F8" r:id="rId7"/>
     <hyperlink ref="F9" r:id="rId8"/>
+    <hyperlink ref="F10" r:id="rId9"/>
+    <hyperlink ref="F11" r:id="rId10"/>
+    <hyperlink ref="F12" r:id="rId11"/>
+    <hyperlink ref="F13" r:id="rId12"/>
+    <hyperlink ref="F14" r:id="rId13"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Add batch 3 to israelis-50-plus database: Pini Shechter (triple jump)
1 new verified row (14 total) - resumed the sport at 50 after decades
away, now world vice-champion for his age category at 78. Also logs
this round's excluded candidates and empty searches per the skill's
running-log convention.
</commit_message>
<xml_diff>
--- a/.claude/skills/israelis-50-plus-database/database.xlsx
+++ b/.claude/skills/israelis-50-plus-database/database.xlsx
@@ -1,17 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="11_573B52B86D4F5BBB7ED903AAEDE48F2C0750C7CF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0FA6FACF-A4B5-43DA-9D15-424765F1FFC2}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="מאגר" state="visible" r:id="rId4"/>
+    <sheet name="מאגר" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="87">
   <si>
     <t>שם</t>
   </si>
@@ -254,24 +258,42 @@
   </si>
   <si>
     <t>https://www.haaretz.co.il/news/local/2025-02-14/ty-article/.premium/00000195-00ec-d1d7-a9d5-f8edb3990000</t>
+  </si>
+  <si>
+    <t>פיני שכטר</t>
+  </si>
+  <si>
+    <t>50 (כיום 78)</t>
+  </si>
+  <si>
+    <t>עבד במשרד, לא עסק בספורט שנים רבות (עסק בקפיצות כנער)</t>
+  </si>
+  <si>
+    <t>בגיל 50 חזר לספורט - קפיצה משולשת; כיום סגן אלוף עולם באתלטיקה לוותיקים בקטגוריית גיל 75-79</t>
+  </si>
+  <si>
+    <t>אתלטיקה - קפיצה משולשת</t>
+  </si>
+  <si>
+    <t>https://www.ynet.co.il/articles/0,7340,L-5332576,00.html</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="12"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="12"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -280,8 +302,8 @@
     </font>
     <font>
       <u/>
+      <sz val="11"/>
       <color rgb="FF0563C1"/>
-      <sz val="11"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -310,7 +332,9 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="medium"/>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -666,9 +690,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F14"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
@@ -678,7 +702,7 @@
     <col min="6" max="6" width="45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -698,7 +722,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -718,7 +742,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -738,7 +762,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>17</v>
       </c>
@@ -758,7 +782,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>21</v>
       </c>
@@ -778,7 +802,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>27</v>
       </c>
@@ -798,7 +822,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>33</v>
       </c>
@@ -818,7 +842,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>39</v>
       </c>
@@ -838,7 +862,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>45</v>
       </c>
@@ -858,7 +882,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>51</v>
       </c>
@@ -878,7 +902,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>57</v>
       </c>
@@ -898,7 +922,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>63</v>
       </c>
@@ -918,7 +942,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>69</v>
       </c>
@@ -938,7 +962,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" ht="57" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>75</v>
       </c>
@@ -958,23 +982,43 @@
         <v>80</v>
       </c>
     </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>81</v>
+      </c>
+      <c r="B15" t="s">
+        <v>82</v>
+      </c>
+      <c r="C15" t="s">
+        <v>83</v>
+      </c>
+      <c r="D15" t="s">
+        <v>84</v>
+      </c>
+      <c r="E15" t="s">
+        <v>85</v>
+      </c>
+      <c r="F15" t="s">
+        <v>86</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1"/>
-    <hyperlink ref="F3" r:id="rId2"/>
-    <hyperlink ref="F4" r:id="rId3"/>
-    <hyperlink ref="F5" r:id="rId4"/>
-    <hyperlink ref="F6" r:id="rId5"/>
-    <hyperlink ref="F7" r:id="rId6"/>
-    <hyperlink ref="F8" r:id="rId7"/>
-    <hyperlink ref="F9" r:id="rId8"/>
-    <hyperlink ref="F10" r:id="rId9"/>
-    <hyperlink ref="F11" r:id="rId10"/>
-    <hyperlink ref="F12" r:id="rId11"/>
-    <hyperlink ref="F13" r:id="rId12"/>
-    <hyperlink ref="F14" r:id="rId13"/>
+    <hyperlink ref="F2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="F3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="F4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="F5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="F6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="F7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="F8" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="F9" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="F10" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="F11" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="F12" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="F13" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="F14" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
50-plus database: add publication-year column, split by 2022, batch 4
Split into two sheets per Leah's request: "כתבות חדשות (2022+)" (4
rows) and "כתבות ישנות (לפני 2022)" (11 rows after adding Esther
Levy - bicycle riding starting at 75). Year verified by direct fetch
for all but one row (Ilan Brosh, mako blocks direct access - flagged
lower-confidence).
</commit_message>
<xml_diff>
--- a/.claude/skills/israelis-50-plus-database/database.xlsx
+++ b/.claude/skills/israelis-50-plus-database/database.xlsx
@@ -3,19 +3,20 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_573B52B86D4F5BBB7ED903AAEDE48F2C0750C7CF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0FA6FACF-A4B5-43DA-9D15-424765F1FFC2}"/>
+  <xr:revisionPtr revIDLastSave="138" documentId="11_573B52B86D4F5BBB7ED903AAEDE48F2C0750C7CF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{74A3489D-05FF-4A8A-ACA2-BAFF0139BF74}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="מאגר" sheetId="1" r:id="rId1"/>
+    <sheet name="כתבות חדשות (2022+)" sheetId="1" r:id="rId1"/>
+    <sheet name="כתבות ישנות (לפני 2022)" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="91">
   <si>
     <t>שם</t>
   </si>
@@ -101,9 +102,6 @@
     <t>ד"ר עמי שינפלד</t>
   </si>
   <si>
-    <t>51</t>
-  </si>
-  <si>
     <t>מנתח לב בכיר בשיבא, אדם יושבני שהיה משוכנע שאינו מסוגל לרוץ</t>
   </si>
   <si>
@@ -155,9 +153,6 @@
     <t>פולינה כצמן</t>
   </si>
   <si>
-    <t>54</t>
-  </si>
-  <si>
     <t>קטועת רגל משמאל (תאונת דרכים בגיל 23), עבדה שנים כמטפלת בקשישים</t>
   </si>
   <si>
@@ -227,9 +222,6 @@
     <t>פסקל ברקוביץ</t>
   </si>
   <si>
-    <t>55</t>
-  </si>
-  <si>
     <t>ספורטאית פראלימפית מנוסה (שחייה מגיל 20, חתירה מגיל 40) שאיבדה את רגליה בתאונה בפריז כשהייתה צעירה</t>
   </si>
   <si>
@@ -276,6 +268,27 @@
   </si>
   <si>
     <t>https://www.ynet.co.il/articles/0,7340,L-5332576,00.html</t>
+  </si>
+  <si>
+    <t>שנת פרסום הכתבה</t>
+  </si>
+  <si>
+    <t>אסתר הלוי</t>
+  </si>
+  <si>
+    <t>כ-75 (כיום כמעט 80)</t>
+  </si>
+  <si>
+    <t>מעולם לא רכבה על אופניים - הוריה לא הרשו לה בילדות</t>
+  </si>
+  <si>
+    <t>התחילה ללמוד לרכוב על אופניים בגיל 75, וממשיכה בשיעורים קבועים</t>
+  </si>
+  <si>
+    <t>רכיבה על אופניים</t>
+  </si>
+  <si>
+    <t>https://xnet.ynet.co.il/articles/0,7340,L-5663476,00.html</t>
   </si>
 </sst>
 </file>
@@ -367,6 +380,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -691,7 +708,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -702,7 +719,7 @@
     <col min="6" max="6" width="45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -721,304 +738,462 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="G1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>6</v>
+        <v>32</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>7</v>
+        <v>33</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+      <c r="G2">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>13</v>
+        <v>39</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+      <c r="G3">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>18</v>
+        <v>67</v>
+      </c>
+      <c r="B4" s="2">
+        <v>55</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>19</v>
+        <v>68</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>20</v>
+        <v>69</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>16</v>
+        <v>70</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+      <c r="G4">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="57" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>21</v>
+        <v>72</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>22</v>
+        <v>73</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>23</v>
+        <v>74</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>24</v>
+        <v>75</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>25</v>
+        <v>76</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="42.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="57" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C14" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>81</v>
-      </c>
-      <c r="B15" t="s">
-        <v>82</v>
-      </c>
-      <c r="C15" t="s">
-        <v>83</v>
-      </c>
-      <c r="D15" t="s">
-        <v>84</v>
-      </c>
-      <c r="E15" t="s">
-        <v>85</v>
-      </c>
-      <c r="F15" t="s">
-        <v>86</v>
-      </c>
+      <c r="G5">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="3"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="3"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="3"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="3"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="3"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="3"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="3"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="3"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="F3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="F4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="F5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="F6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="F7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="F8" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="F9" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="F10" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="F11" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="F12" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="F13" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="F14" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7754BC0-AB45-43C0-8845-99EFF23F68F7}">
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2">
+        <v>2016</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3">
+        <v>2016</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4">
+        <v>2016</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6">
+        <v>51</v>
+      </c>
+      <c r="C6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G6">
+        <v>2013</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7">
+        <v>54</v>
+      </c>
+      <c r="C7" t="s">
+        <v>45</v>
+      </c>
+      <c r="D7" t="s">
+        <v>46</v>
+      </c>
+      <c r="E7" t="s">
+        <v>47</v>
+      </c>
+      <c r="F7" t="s">
+        <v>48</v>
+      </c>
+      <c r="G7">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8" t="s">
+        <v>51</v>
+      </c>
+      <c r="D8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E8" t="s">
+        <v>53</v>
+      </c>
+      <c r="F8" t="s">
+        <v>54</v>
+      </c>
+      <c r="G8">
+        <v>2013</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9" t="s">
+        <v>56</v>
+      </c>
+      <c r="C9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D9" t="s">
+        <v>58</v>
+      </c>
+      <c r="E9" t="s">
+        <v>59</v>
+      </c>
+      <c r="F9" t="s">
+        <v>60</v>
+      </c>
+      <c r="G9">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" t="s">
+        <v>63</v>
+      </c>
+      <c r="D10" t="s">
+        <v>64</v>
+      </c>
+      <c r="E10" t="s">
+        <v>65</v>
+      </c>
+      <c r="F10" t="s">
+        <v>66</v>
+      </c>
+      <c r="G10">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>78</v>
+      </c>
+      <c r="B11" t="s">
+        <v>79</v>
+      </c>
+      <c r="C11" t="s">
+        <v>80</v>
+      </c>
+      <c r="D11" t="s">
+        <v>81</v>
+      </c>
+      <c r="E11" t="s">
+        <v>82</v>
+      </c>
+      <c r="F11" t="s">
+        <v>83</v>
+      </c>
+      <c r="G11">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>85</v>
+      </c>
+      <c r="B12" t="s">
+        <v>86</v>
+      </c>
+      <c r="C12" t="s">
+        <v>87</v>
+      </c>
+      <c r="D12" t="s">
+        <v>88</v>
+      </c>
+      <c r="E12" t="s">
+        <v>89</v>
+      </c>
+      <c r="F12" t="s">
+        <v>90</v>
+      </c>
+      <c r="G12">
+        <v>2020</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>